<commit_message>
feat(F-NAR-019): ATOM-COL.POL.001-04 La tomate de Victorina
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.POL.001-04.xlsx
+++ b/stories/arbres/ATOM-COL.POL.001-04.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>La tomate tiède de Victorina</t>
+          <t>La tomate de Victorina</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>marché au soleil, caisses de tomates</t>
+          <t>marché au soleil, bâche rayée, caisses, tomates, terre et sucré, sac de toile</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Victorina veut la tomate ronde au bord de la caisse. Elle dit bonjour, s'il te plaît, merci. La tomate reste tiède.</t>
+          <t>Un claquement court. Sur la toile, un éclat de bâche luit. Victorina veut la tomate lisse maintenant. Elle tend la main trop vite, sans le mot : le marchand n'a pas les yeux. Elle refuse de foncer, dit bonjour, s'il te plaît, obtient la tomate. Merci vécu. Le sac glisse, la tomate penche. Elle refuse, tient des deux mains. Un éclat de bâche reste pâle.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le soleil chauffe le bois des caisses. Une feuille de tomate colle à une sandale. Ça sent la terre, un peu sucrée. Une bâche rayée claque au-dessus. Le sac de papa est en toile grise. Il pend à son épaule. Tu as vu le rouge, Victorina ? Elles sont rouges, maman. Bien rouges. Les pavés sont encore un peu humides. Une mouche tourne près d'une feuille. Maman tient un panier d'osier. L'osier gratte un peu le manteau. Tu sens la terre, Victorina ? Oui, papa. C'est sucré un peu. En ce moment, Victorina s'arrête. Une tomate lisse brille au bord. Elle est ronde. Elle est un peu tiède. Je la veux, papa. Tu restes près de nous. Le marchand essuie une caisse. Le bois est clair, un peu rêche. Victorina se tient près de maman. Il a le chiffon à la main. On le laisse finir. Le chiffon se pose sur le bois. Le marchand lève la tête. Victorina montre la tomate ronde. Tu demandes, Victorina.</t>
+          <t>Un claquement court au-dessus des caisses. La bâche rayée se tend, puis relâche. Sur la toile, un éclat de bâche luit. Il brille, papa. Tu le vois, sur la toile ? Victorina touche la toile, un instant. La toile est chaude sous le doigt. Elle est chaude. Le soleil tient sur les caisses. Voilà. Le soleil pique un peu les bras. J'ai les bras chauds. On reste sous la bâche. Tu as de l'ombre, là. Oui, maman. Une odeur de terre arrive. Elle sent le sucré aussi. Ça sent le jardin ! Tu sens, Victorina ? Oui. Le sac de papa pend à l'épaule. Le sac est en toile grise. On marche près des caisses. Tu restes près de nous ? Oui, maman. Une mouche tourne près d'une feuille. Une flaque tient un morceau de ciel. Le ciel est dans l'eau. Oui. Une balance de fer attend. Le bois des caisses est clair. En ce moment, Victorina s'arrête devant l'étal. Une tomate lisse brille au bord. Elle est ronde. Elle est un peu tiède. Je la veux, maintenant. Victorina tend la main trop vite. Les doigts touchent le bois rêche. Celle-là ! Sa voix se mélange au marché. Le marchand essuie une caisse. Il n'a pas levé les yeux. Oh. La tomate reste sur le bois. L'éclat de bâche tremble, puis tient. Le sourire de Victorina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je la prends ! La tomate est sur le bois. Tu la vois, Victorina ? Les épaules de Victorina tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur. Tu parles au marchand, Victorina ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le soleil chauffe le bois des caisses. Une feuille de tomate colle à une sandale. Ça sent la terre, un peu sucrée. Une bâche rayée claque au-dessus. Le sac de papa est en toile grise. Il pend à son épaule. Tu as vu le rouge, Victorina ? Elles sont rouges, maman. Bien rouges. Les pavés sont encore un peu humides. Une mouche tourne près d'une feuille. Maman tient un panier d'osier. L'osier gratte un peu le manteau. Tu sens la terre, Victorina ? Oui, papa. C'est sucré un peu. En ce moment, Victorina s'arrête. Une tomate lisse brille au bord. Elle est ronde. Elle est un peu tiède. Je la veux, papa. Tu restes près de nous. Le marchand essuie une caisse. Le bois est clair, un peu rêche. Victorina se tient près de maman. Il a le chiffon à la main. On le laisse finir. Le chiffon se pose sur le bois. Le marchand lève la tête. Victorina montre la tomate ronde. Tu demandes, Victorina.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un claquement court au-dessus des caisses. La bâche rayée se tend, puis relâche. Sur la toile, un &lt;emphasis level="moderate"&gt;éclat de bâche&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, sur la toile ? Victorina touche la toile, un instant. La toile est chaude sous le doigt. Elle est chaude. Le soleil tient sur les caisses. Voilà. Le soleil pique un peu les bras. J'ai les bras chauds. On reste sous la bâche. Tu as de l'ombre, là. Oui, maman. Une odeur de terre arrive. Elle sent le sucré aussi. Ça sent le jardin ! Tu sens, Victorina ? Oui. Le sac de papa pend à l'épaule. Le sac est en toile grise. On marche près des caisses. Tu restes près de nous ? Oui, maman. Une mouche tourne près d'une feuille. Une flaque tient un morceau de ciel. Le ciel est dans l'eau. Oui. Une balance de fer attend. Le bois des caisses est clair. En ce moment, Victorina s'arrête devant l'étal. Une tomate lisse brille au bord. Elle est ronde. Elle est un peu tiède. Je la veux, maintenant. Victorina tend la main trop vite. Les doigts touchent le bois rêche. Celle-là ! Sa voix se mélange au marché. Le marchand essuie une caisse. Il n'a pas levé les yeux. Oh. La tomate reste sur le bois. L'éclat de bâche tremble, puis tient. Le sourire de Victorina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je la prends ! La tomate est sur le bois. Tu la vois, Victorina ? Les épaules de Victorina tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur. Tu parles au marchand, Victorina ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lucien va au marché avec papa. Les étals sentent les tomates. Lucien voit le marchand. Papa dit : on salue. Lucien dit : &lt;emphasis&gt;bonjour&lt;/emphasis&gt;. Le marchand sourit. Lucien veut une tomate. Papa dit : on demande. Lucien dit : une tomate, s'il te plaît. Le marchand tend la tomate. Elle est lisse. Lucien dit : merci. Papa sourit. On dit bonjour. On dit s'il te plaît. On dit merci. Lucien touche la tomate. Elle est un peu tiède. Le marchand dit : au revoir. Lucien répète : bonjour. S'il te plaît. Merci.&lt;/slow&gt; [pause]</t>
+          <t>Un claquement court au-dessus des caisses. La bâche rayée se tend, puis relâche. Sur la toile, un &lt;emphasis&gt;éclat de bâche&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, sur la toile ? Victorina touche la toile, un instant. La toile est chaude sous le doigt. Elle est chaude. Le soleil tient sur les caisses. Voilà. Le soleil pique un peu les bras. J'ai les bras chauds. On reste sous la bâche. Tu as de l'ombre, là. Oui, maman. Une odeur de terre arrive. Elle sent le sucré aussi. Ça sent le jardin ! Tu sens, Victorina ? Oui. Le sac de papa pend à l'épaule. Le sac est en toile grise. On marche près des caisses. Tu restes près de nous ? Oui, maman. Une mouche tourne près d'une feuille. Une flaque tient un morceau de ciel. Le ciel est dans l'eau. Oui. Une balance de fer attend. Le bois des caisses est clair. En ce moment, Victorina s'arrête devant l'étal. Une tomate lisse brille au bord. Elle est ronde. Elle est un peu tiède. Je la veux, maintenant. Victorina tend la main trop vite. Les doigts touchent le bois rêche. Celle-là ! Sa voix se mélange au marché. Le marchand essuie une caisse. Il n'a pas levé les yeux. Oh. La tomate reste sur le bois. L'éclat de bâche tremble, puis tient. Le sourire de Victorina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je la prends ! La tomate est sur le bois. Tu la vois, Victorina ? Les épaules de Victorina tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur. Tu parles au marchand, Victorina ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,18 +1246,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>bonjour</t>
+          <t>éclat de bâche</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,47 +1324,74 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_la_tomate_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le soleil chauffe le bois des caisses.
-narrateur|Une feuille de tomate colle à une sandale.
-narrateur|Ça sent la terre, un peu sucrée.
-narrateur|Une bâche rayée claque au-dessus.
-narrateur|Le sac de papa est en toile grise.
-narrateur|Il pend à son épaule.
-maman|Tu as vu le rouge, Victorina ?
-enfant-f|Elles sont rouges, maman.
-papa|Bien rouges.
-narrateur|Les pavés sont encore un peu humides.
+          <t>narrateur|Un claquement court au-dessus des caisses.
+narrateur|La bâche rayée se tend, puis relâche.
+narrateur|Sur la toile, un éclat de bâche luit.
+enfant-f|Il brille, papa.
+papa|Tu le vois, sur la toile ?
+narrateur|Victorina touche la toile, un instant.
+narrateur|La toile est chaude sous le doigt.
+enfant-f|Elle est chaude.
+maman|Le soleil tient sur les caisses.
+papa|Voilà.
+narrateur|Le soleil pique un peu les bras.
+enfant-f|J'ai les bras chauds.
+papa|On reste sous la bâche.
+maman|Tu as de l'ombre, là.
+enfant-f|Oui, maman.
+narrateur|Une odeur de terre arrive.
+narrateur|Elle sent le sucré aussi.
+enfant-f|Ça sent le jardin !
+maman|Tu sens, Victorina ?
+enfant-f|Oui.
+narrateur|Le sac de papa pend à l'épaule.
+narrateur|Le sac est en toile grise.
+papa|On marche près des caisses.
+maman|Tu restes près de nous ?
+enfant-f|Oui, maman.
 narrateur|Une mouche tourne près d'une feuille.
-narrateur|Maman tient un panier d'osier.
-narrateur|L'osier gratte un peu le manteau.
-papa|Tu sens la terre, Victorina ?
-enfant-f|Oui, papa.
-enfant-f|C'est sucré un peu.
-narrateur|En ce moment, Victorina s'arrête.
+narrateur|Une flaque tient un morceau de ciel.
+enfant-f|Le ciel est dans l'eau.
+papa|Oui.
+narrateur|Une balance de fer attend.
+narrateur|Le bois des caisses est clair.
+narrateur|En ce moment, Victorina s'arrête devant l'étal.
 narrateur|Une tomate lisse brille au bord.
 narrateur|Elle est ronde.
 narrateur|Elle est un peu tiède.
-enfant-f|Je la veux, papa.
-papa|Tu restes près de nous.
+enfant-f|Je la veux, maintenant.
+narrateur|Victorina tend la main trop vite.
+narrateur|Les doigts touchent le bois rêche.
+enfant-f|Celle-là !
+narrateur|Sa voix se mélange au marché.
 narrateur|Le marchand essuie une caisse.
-narrateur|Le bois est clair, un peu rêche.
-narrateur|Victorina se tient près de maman.
-maman|Il a le chiffon à la main.
-papa|On le laisse finir.
-narrateur|Le chiffon se pose sur le bois.
-narrateur|Le marchand lève la tête.
-narrateur|Victorina montre la tomate ronde.
-maman|Tu demandes, Victorina.</t>
+narrateur|Il n'a pas levé les yeux.
+enfant-f|Oh.
+narrateur|La tomate reste sur le bois.
+narrateur|L'éclat de bâche tremble, puis tient.
+narrateur|Le sourire de Victorina disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-f|Je la prends !
+maman|La tomate est sur le bois.
+papa|Tu la vois, Victorina ?
+narrateur|Les épaules de Victorina tombent un peu.
+narrateur|Ça serre, dans son ventre.
+narrateur|Papa se baisse à sa hauteur.
+papa|Tu parles au marchand, Victorina ?</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>marche,bache</t>
+          <t>bache,caisse</t>
         </is>
       </c>
     </row>
@@ -1391,17 +1418,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Victorina veut la tomate. Que dit-elle ?</t>
+          <t>Victorina parle au marchand. Quels mots dit-elle ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Victorina veut la tomate. Que dit-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Victorina parle au &lt;emphasis level="moderate"&gt;marchand&lt;/emphasis&gt;. Quels mots dit-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lucien parle au marchand. Quels mots dit-il ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Victorina parle au &lt;emphasis&gt;marchand&lt;/emphasis&gt;. Quels mots dit-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1426,7 +1453,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Elle dit bonjour. Que dit Victorina ?</t>
+          <t>Elle dit bonjour. Quels mots dit Victorina ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1464,7 +1491,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1472,10 +1499,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1490,34 +1517,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>marchand</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1526,13 +1557,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1542,13 +1573,13 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_dit_bonjour_au_marchand; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Victorina veut la tomate.
-narrateur|Que dit-elle ?</t>
+          <t>narrateur|Victorina parle au marchand.
+narrateur|Quels mots dit-elle ?</t>
         </is>
       </c>
     </row>
@@ -1575,17 +1606,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. Une tomate, s'il te plaît. Celle du bord. Le marchand pose la tomate. Elle est dans la main de Victorina. Elle est lisse. Elle est tiède. Elle sent le jardin. Merci. Merci. Elle est douce, papa. Oui. Tu la mets dans le sac ? Oui, maman. Papa ouvre le sac de toile. Victorina pose la tomate au fond. Le sac sent le pain d'hier. Tu tiens le bord ? Oui. La bâche claque encore. Une goutte brille sur la tomate. On rentre tout doux.</t>
+          <t>Victorina avance trop vite vers le bois. Celle-là, maintenant ! Sa voix se mélange aux caisses. Oh. La tomate reste sur le bois. Elle refuse de foncer. Victorina referme la main. Elle écoute la bâche, un instant. Tu veux venir près du bois ? Papa s'accroupit à la même hauteur. Victorina pose un pied près de la caisse. Le bois est tiède, un peu rêche. Celle-là. Bonjour. Bonjour. Une tomate, s'il te plaît. Le marchand lève enfin les yeux. Derrière le bois, une main se tend. La tomate passe dans la paume. Merci. Merci, Victorina. Papa a entendu toute la phrase. Le ventre de Victorina se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Ça sent la terre et le sucré. La tomate est à moi. Elle est dans tes mains. Victorina pose une main sur la tomate. La peau est lisse, un peu tiède. Tu la mets dans le sac ? Oui, papa. Papa ouvre le sac de toile. Victorina pose la tomate au fond. Le sac sent la toile chaude.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. Une tomate, s'il te plaît. Celle du bord. Le marchand pose la tomate. Elle est dans la main de Victorina. Elle est lisse. Elle est tiède. Elle sent le jardin. Merci. Merci. Elle est douce, papa. Oui. Tu la mets dans le sac ? Oui, maman. Papa ouvre le sac de toile. Victorina pose la tomate au fond. Le sac sent le pain d'hier. Tu tiens le bord ? Oui. La bâche claque encore. Une goutte brille sur la tomate. On rentre tout doux.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorina avance trop vite vers le bois. Celle-là, maintenant ! Sa voix se mélange aux caisses. Oh. La tomate reste sur le bois. Elle refuse de foncer. Victorina referme la main. Elle écoute la bâche, un instant. Tu veux venir près du bois ? Papa s'accroupit à la même hauteur. Victorina pose un pied près de la caisse. Le bois est tiède, un peu rêche. Celle-là. Bonjour. Bonjour. Une tomate, s'il te plaît. Le marchand lève enfin les yeux. Derrière le bois, une main se tend. La tomate passe dans la paume. Merci. Merci, Victorina. Papa a entendu toute la phrase. Le ventre de Victorina se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Ça sent la terre et le sucré. La tomate est à moi. Elle est dans tes mains. Victorina pose une main sur la tomate. La peau est lisse, un peu tiède. Tu la mets dans le sac ? Oui, papa. Papa ouvre le sac de toile. Victorina pose la tomate au fond. Le sac sent la toile chaude.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lucien a dit &lt;emphasis&gt;bonjour&lt;/emphasis&gt;. Puis s'il te plaît. Puis merci. Papa était là.&lt;/slow&gt; [pause]</t>
+          <t>Victorina avance trop vite vers le bois. Celle-là, maintenant ! Sa voix se mélange aux caisses. Oh. La tomate reste sur le bois. Elle refuse de foncer. Victorina referme la main. Elle écoute la bâche, un instant. Tu veux venir près du bois ? Papa s'accroupit à la même hauteur. Victorina pose un pied près de la caisse. Le bois est tiède, un peu rêche. Celle-là. Bonjour. Bonjour. Une tomate, s'il te plaît. Le marchand lève enfin les yeux. Derrière le bois, une main se tend. La tomate passe dans la paume. Merci. Merci, Victorina. Papa a entendu toute la phrase. Le ventre de Victorina se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Ça sent la terre et le sucré. La tomate est à moi. Elle est dans tes mains. Victorina pose une main sur la tomate. La peau est lisse, un peu tiède. Tu la mets dans le sac ? Oui, papa. Papa ouvre le sac de toile. Victorina pose la tomate au fond. Le sac sent la toile chaude. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1632,18 +1663,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1676,20 +1707,20 @@
         <v>450</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>280</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1698,10 +1729,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1710,43 +1741,56 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=soulagement_prudent; intensite=1; destinataire=enfant; sous_texte=la_main_echoue_le_mot_ouvre; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>enfant-f|Bonjour.
+          <t>narrateur|Victorina avance trop vite vers le bois.
+enfant-f|Celle-là, maintenant !
+narrateur|Sa voix se mélange aux caisses.
+enfant-f|Oh.
+narrateur|La tomate reste sur le bois.
+narrateur|Elle refuse de foncer.
+narrateur|Victorina referme la main.
+narrateur|Elle écoute la bâche, un instant.
+papa|Tu veux venir près du bois ?
+narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Victorina pose un pied près de la caisse.
+narrateur|Le bois est tiède, un peu rêche.
+enfant-f|Celle-là.
+enfant-f|Bonjour.
 papa|Bonjour.
 enfant-f|Une tomate, s'il te plaît.
-enfant-f|Celle du bord.
-narrateur|Le marchand pose la tomate.
-narrateur|Elle est dans la main de Victorina.
-narrateur|Elle est lisse.
-narrateur|Elle est tiède.
-narrateur|Elle sent le jardin.
+narrateur|Le marchand lève enfin les yeux.
+narrateur|Derrière le bois, une main se tend.
+narrateur|La tomate passe dans la paume.
 enfant-f|Merci.
-maman|Merci.
-enfant-f|Elle est douce, papa.
-papa|Oui.
-maman|Tu la mets dans le sac ?
-enfant-f|Oui, maman.
+papa|Merci, Victorina.
+narrateur|Papa a entendu toute la phrase.
+narrateur|Le ventre de Victorina se desserre.
+narrateur|Les épaules se relèvent un peu.
+maman|Tu as les mains au chaud ?
+enfant-f|Un peu, maman.
+narrateur|Ça sent la terre et le sucré.
+enfant-f|La tomate est à moi.
+maman|Elle est dans tes mains.
+narrateur|Victorina pose une main sur la tomate.
+narrateur|La peau est lisse, un peu tiède.
+papa|Tu la mets dans le sac ?
+enfant-f|Oui, papa.
 narrateur|Papa ouvre le sac de toile.
 narrateur|Victorina pose la tomate au fond.
-narrateur|Le sac sent le pain d'hier.
-papa|Tu tiens le bord ?
-enfant-f|Oui.
-narrateur|La bâche claque encore.
-narrateur|Une goutte brille sur la tomate.
-maman|On rentre tout doux.</t>
+narrateur|Le sac sent la toile chaude.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>sac</t>
+          <t>caisse,sac</t>
         </is>
       </c>
     </row>
@@ -1773,17 +1817,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Ils rentrent par la rue étroite. Les pavés sonnent sous les chaussures. Victorina tient encore le bord du sac. La feuille a quitté la sandale. À la maison, papa lave la tomate. L'eau fait un petit bruit. Tu veux un bout ? Oui, maman. S'il te plaît. Victorina croque un bout. C'est doux. C'est un peu sucré. Merci, Victorina. Merci, maman. Merci, Victorina. Une graine reste sur la table. On la met de côté. La tomate était tiède. Oui. Comme au marché. Le sac de toile repose près de l'évier.</t>
+          <t>Victorina tire le sac trop vite. Je la mange, d'un coup ! Le sac glisse entre les doigts. La tomate penche vers le sol. Oh. Victorina avance les mains. Puis elle s'arrête net. Attends, je regarde. Papa attend, sans parler. Personne ne parle. Victorina refuse de foncer. Elle observe la tomate, un instant. Elle écoute le claquement de la bâche. Sur la toile, un éclat de bâche luit. Là, près de la bâche. Victorina tient le sac des deux mains. La toile est rêche, un peu chaude. Elle est tiède, papa. Tu la portes jusqu'à la rue ? Oui, papa. On sort ? Oui, maman. Ils marchent entre les étals. Une feuille rouge colle à une chaussure. On la laisse, celle-là. Elle n'est pas une tomate. Non. Juste une feuille. Je la tiens. On avance. Victorina serre le sac contre elle. Elle reste tiède. On marche. Le sac penche, puis se cale. Je la tiens bien.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Ils rentrent par la rue étroite. Les pavés sonnent sous les chaussures. Victorina tient encore le bord du sac. La feuille a quitté la sandale. À la maison, papa lave la tomate. L'eau fait un petit bruit. Tu veux un bout ? Oui, maman. S'il te plaît. Victorina croque un bout. C'est doux. C'est un peu sucré. Merci, Victorina. Merci, maman. Merci, Victorina. Une graine reste sur la table. On la met de côté. La tomate était tiède. Oui. Comme au marché. Le sac de toile repose près de l'évier.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorina tire le sac trop vite. Je la mange, d'un coup ! Le sac glisse entre les doigts. La tomate penche vers le sol. Oh. Victorina avance les mains. Puis elle s'arrête net. Attends, je regarde. Papa attend, sans parler. Personne ne parle. Victorina refuse de foncer. Elle observe la tomate, un instant. Elle écoute le claquement de la bâche. Sur la toile, un &lt;emphasis level="moderate"&gt;éclat de bâche&lt;/emphasis&gt; luit. Là, près de la bâche. Victorina tient le sac des deux mains. La toile est rêche, un peu chaude. Elle est tiède, papa. Tu la portes jusqu'à la rue ? Oui, papa. On sort ? Oui, maman. Ils marchent entre les étals. Une feuille rouge colle à une chaussure. On la laisse, celle-là. Elle n'est pas une tomate. Non. Juste une feuille. Je la tiens. On avance. Victorina serre le sac contre elle. Elle reste tiède. On marche. Le sac penche, puis se cale. Je la tiens bien.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lucien tient la tomate. Papa dit &lt;emphasis&gt;merci&lt;/emphasis&gt; aussi.&lt;/slow&gt; [pause]</t>
+          <t>Victorina tire le sac trop vite. Je la mange, d'un coup ! Le sac glisse entre les doigts. La tomate penche vers le sol. Oh. Victorina avance les mains. Puis elle s'arrête net. Attends, je regarde. Papa attend, sans parler. Personne ne parle. Victorina refuse de foncer. Elle observe la tomate, un instant. Elle écoute le claquement de la bâche. Sur la toile, un &lt;emphasis&gt;éclat de bâche&lt;/emphasis&gt; luit. Là, près de la bâche. Victorina tient le sac des deux mains. La toile est rêche, un peu chaude. Elle est tiède, papa. Tu la portes jusqu'à la rue ? Oui, papa. On sort ? Oui, maman. Ils marchent entre les étals. Une feuille rouge colle à une chaussure. On la laisse, celle-là. Elle n'est pas une tomate. Non. Juste une feuille. Je la tiens. On avance. Victorina serre le sac contre elle. Elle reste tiède. On marche. Le sac penche, puis se cale. Je la tiens bien. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1830,18 +1874,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1864,30 +1908,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>merci</t>
+          <t>éclat de bâche</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1896,10 +1940,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1908,37 +1952,55 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_sans_regarder_l_eclat; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Ils rentrent par la rue étroite.
-narrateur|Les pavés sonnent sous les chaussures.
-narrateur|Victorina tient encore le bord du sac.
-narrateur|La feuille a quitté la sandale.
-narrateur|À la maison, papa lave la tomate.
-narrateur|L'eau fait un petit bruit.
-maman|Tu veux un bout ?
+          <t>narrateur|Victorina tire le sac trop vite.
+enfant-f|Je la mange, d'un coup !
+narrateur|Le sac glisse entre les doigts.
+narrateur|La tomate penche vers le sol.
+enfant-f|Oh.
+narrateur|Victorina avance les mains.
+narrateur|Puis elle s'arrête net.
+enfant-f|Attends, je regarde.
+narrateur|Papa attend, sans parler.
+narrateur|Personne ne parle.
+narrateur|Victorina refuse de foncer.
+narrateur|Elle observe la tomate, un instant.
+narrateur|Elle écoute le claquement de la bâche.
+narrateur|Sur la toile, un éclat de bâche luit.
+enfant-f|Là, près de la bâche.
+narrateur|Victorina tient le sac des deux mains.
+narrateur|La toile est rêche, un peu chaude.
+enfant-f|Elle est tiède, papa.
+papa|Tu la portes jusqu'à la rue ?
+enfant-f|Oui, papa.
+maman|On sort ?
 enfant-f|Oui, maman.
-enfant-f|S'il te plaît.
-narrateur|Victorina croque un bout.
-enfant-f|C'est doux.
-enfant-f|C'est un peu sucré.
-maman|Merci, Victorina.
-enfant-f|Merci, maman.
-papa|Merci, Victorina.
-narrateur|Une graine reste sur la table.
-maman|On la met de côté.
-enfant-f|La tomate était tiède.
-papa|Oui.
-papa|Comme au marché.
-narrateur|Le sac de toile repose près de l'évier.</t>
+narrateur|Ils marchent entre les étals.
+narrateur|Une feuille rouge colle à une chaussure.
+papa|On la laisse, celle-là.
+enfant-f|Elle n'est pas une tomate.
+papa|Non.
+maman|Juste une feuille.
+enfant-f|Je la tiens.
+maman|On avance.
+narrateur|Victorina serre le sac contre elle.
+enfant-f|Elle reste tiède.
+papa|On marche.
+narrateur|Le sac penche, puis se cale.
+enfant-f|Je la tiens bien.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>eau</t>
+          <t>sac,marche</t>
         </is>
       </c>
     </row>
@@ -1965,17 +2027,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Il reste un bout, bien rouge. La graine attend sur la table. Bonne journée, Victorina. Elle était ronde, ta tomate.</t>
+          <t>La bâche brillait, papa. Tu le vois, comme au marché ? Oui, sur la toile. Victorina pose le sac contre elle. On la garde au chaud ? Oui, maman. Les tomates sentaient bon. Elle est contre toi. Une odeur de terre monte du sac. Victorina respire, plus large. On rentre ? Oui. Les joues de Victorina se réchauffent. Le sac reste tiède sous la main. On le voit, maman. Tu le vois sur la toile ? Oui, l'éclat. Un éclat de bâche reste pâle.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Il reste un bout, bien rouge. La graine attend sur la table. Bonne journée, Victorina. Elle était ronde, ta tomate.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La bâche brillait, papa. Tu le vois, comme au marché ? Oui, sur la toile. Victorina pose le sac contre elle. On la garde au chaud ? Oui, maman. Les tomates sentaient bon. Elle est contre toi. Une odeur de terre monte du sac. Victorina respire, plus large. On rentre ? Oui. Les joues de Victorina se réchauffent. Le sac reste tiède sous la main. On le voit, maman. Tu le vois sur la toile ? Oui, l'éclat. Un &lt;emphasis level="moderate"&gt;éclat de bâche&lt;/emphasis&gt; reste pâle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La bâche brillait, papa. Tu le vois, comme au marché ? Oui, sur la toile. Victorina pose le sac contre elle. On la garde au chaud ? Oui, maman. Les tomates sentaient bon. Elle est contre toi. Une odeur de terre monte du sac. Victorina respire, plus large. On rentre ? Oui. Les joues de Victorina se réchauffent. Le sac reste tiède sous la main. On le voit, maman. Tu le vois sur la toile ? Oui, l'éclat. Un &lt;emphasis&gt;éclat de bâche&lt;/emphasis&gt; reste pâle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2022,7 +2084,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2030,10 +2092,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.36</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2042,12 +2104,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2056,17 +2118,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de bâche</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2075,11 +2141,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2088,27 +2154,50 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_pale; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Il reste un bout, bien rouge.
-narrateur|La graine attend sur la table.
-maman|Bonne journée, Victorina.
-papa|Elle était ronde, ta tomate.</t>
+          <t>enfant-f|La bâche brillait, papa.
+papa|Tu le vois, comme au marché ?
+enfant-f|Oui, sur la toile.
+narrateur|Victorina pose le sac contre elle.
+maman|On la garde au chaud ?
+enfant-f|Oui, maman.
+enfant-f|Les tomates sentaient bon.
+maman|Elle est contre toi.
+narrateur|Une odeur de terre monte du sac.
+narrateur|Victorina respire, plus large.
+papa|On rentre ?
+enfant-f|Oui.
+narrateur|Les joues de Victorina se réchauffent.
+narrateur|Le sac reste tiède sous la main.
+enfant-f|On le voit, maman.
+maman|Tu le vois sur la toile ?
+enfant-f|Oui, l'éclat.
+narrateur|Un éclat de bâche reste pâle.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>bache</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2221,6 +2310,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>